<commit_message>
new client culture tggrt
</commit_message>
<xml_diff>
--- a/anydesk.xlsx
+++ b/anydesk.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="74">
   <si>
     <t>Direction</t>
   </si>
@@ -509,14 +509,14 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -798,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BF36"/>
+  <dimension ref="A1:BF37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -2486,6 +2486,34 @@
       <c r="K36" s="11"/>
       <c r="L36" s="3"/>
     </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A37" s="21">
+        <v>34</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" s="21">
+        <v>1761783449</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F37" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="G37" s="21"/>
+      <c r="H37" s="21"/>
+      <c r="I37" s="21">
+        <v>46326</v>
+      </c>
+      <c r="J37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
+    </row>
   </sheetData>
   <autoFilter ref="C1:C36"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3401,32 +3429,32 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44"/>
       <c r="D16" s="28">
         <f>SUM(D1:D14)</f>
         <v>600000</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A18" s="42" t="s">
+      <c r="A18" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="42"/>
-      <c r="C18" s="42"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
       <c r="D18" s="26">
         <v>10000</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="42" t="s">
+      <c r="A20" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="42"/>
-      <c r="C20" s="42"/>
+      <c r="B20" s="44"/>
+      <c r="C20" s="44"/>
       <c r="D20" s="28">
         <f>D16-D18</f>
         <v>590000</v>
@@ -3468,16 +3496,16 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="43">
+      <c r="A2" s="42">
         <v>2</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="44">
+      <c r="D2" s="43">
         <v>0</v>
       </c>
     </row>
@@ -3805,11 +3833,11 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="42"/>
+      <c r="B28" s="44"/>
+      <c r="C28" s="44"/>
       <c r="D28" s="28">
         <f>D26+D24</f>
         <v>720000</v>
@@ -3884,32 +3912,32 @@
       </c>
     </row>
     <row r="42" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A42" s="42" t="s">
+      <c r="A42" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="B42" s="42"/>
-      <c r="C42" s="42"/>
+      <c r="B42" s="44"/>
+      <c r="C42" s="44"/>
       <c r="D42" s="28">
         <f>SUM(D3:D40)</f>
         <v>2100000</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A44" s="42" t="s">
+      <c r="A44" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="B44" s="42"/>
-      <c r="C44" s="42"/>
+      <c r="B44" s="44"/>
+      <c r="C44" s="44"/>
       <c r="D44" s="26">
         <v>10000</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A46" s="42" t="s">
+      <c r="A46" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="B46" s="42"/>
-      <c r="C46" s="42"/>
+      <c r="B46" s="44"/>
+      <c r="C46" s="44"/>
       <c r="D46" s="28">
         <f>D42-D44</f>
         <v>2090000</v>

</xml_diff>